<commit_message>
fix: remove FormulaRule do openpyxl para evitar corrupção no Drive/Excel
FormulaRule causava aviso de reparo no Excel e falha no visualizador do
Google Drive. Coloração de linhas ATRASADO já era feita via loop Python
direto (c.fill), tornando o FormulaRule redundante e prejudicial.

https://claude.ai/code/session_016vsXRB1Z1r283TkGCSjczo
</commit_message>
<xml_diff>
--- a/Restricoes_Consolidadas_Cristalia_19052026.xlsx
+++ b/Restricoes_Consolidadas_Cristalia_19052026.xlsx
@@ -372,16 +372,6 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
-          <bgColor rgb="00FFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -3666,11 +3656,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M52"/>
-  <conditionalFormatting sqref="A2:M52">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$L2="ATRASADO"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>